<commit_message>
add requested journal feeds
</commit_message>
<xml_diff>
--- a/config/monthly/source对应表.xlsx
+++ b/config/monthly/source对应表.xlsx
@@ -397,7 +397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="66.77734375" customWidth="1" min="1" max="1"/>
@@ -896,6 +896,210 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Recent Articles in Phys. Rev. Lett.</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>APS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Physical Review Letters</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ScienceDirect Publication: Physics Letters B</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Physics Letters B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ACS Applied Materials &amp; Interfaces: Latest Articles (ACS Publications)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ACS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ACS Applied Materials &amp; Interfaces</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nuclear Fusion - latest papers</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>IOP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Nuclear Fusion</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Recent Articles in Phys. Rev. C</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>APS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Physical Review C</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Industrial Informatics - new TOC</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Industrial Informatics</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Sustainable Energy - new TOC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Sustainable Energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Energy Conversion - new TOC</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Energy Conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Smart Grid - new TOC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Smart Grid</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Systems - new TOC</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Delivery - new TOC</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Power Delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nano-Micro Letters</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Springer-Nature</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nano-Micro Letters</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>